<commit_message>
sửa file input excel fine-tuning
</commit_message>
<xml_diff>
--- a/fine_tuning_excel_pack_brand_voice/04_eval_scorecard_UTF8_FIXED.xlsx
+++ b/fine_tuning_excel_pack_brand_voice/04_eval_scorecard_UTF8_FIXED.xlsx
@@ -8,83 +8,127 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\baitap\NT114\NT114-Git\NT114.Q21-Web-Copy-Writing\fine_tuning_excel_pack_brand_voice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0442DDF7-17B7-4640-914D-7BAF8DBAF4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BCFA5978-54F2-4789-AC91-A2079C254206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2244" yWindow="2052" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2244" yWindow="2052" windowWidth="17280" windowHeight="8880" xr2:uid="{66ECA6B2-FAE0-4292-860D-642FA321AAE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Scorecard" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
-  <si>
-    <t>criterion</t>
-  </si>
-  <si>
-    <t>check</t>
-  </si>
-  <si>
-    <t>expected</t>
-  </si>
-  <si>
-    <t>status</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>Pass criteria</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
   <si>
     <t>Prompt contract</t>
   </si>
   <si>
-    <t>Generator UI prompt</t>
-  </si>
-  <si>
-    <t>No TYPE schema</t>
-  </si>
-  <si>
-    <t>pass</t>
-  </si>
-  <si>
-    <t>Vietnamese encoding</t>
-  </si>
-  <si>
-    <t>No replacement question marks in Vietnamese prompt</t>
-  </si>
-  <si>
-    <t>UTF-8</t>
-  </si>
-  <si>
-    <t>Output format</t>
-  </si>
-  <si>
-    <t>Version labels 1-3</t>
-  </si>
-  <si>
-    <t>3 separate versions</t>
+    <t>Mỗi prompt bắt đầu bằng "Bạn là chuyên gia copywriting..." và có block Phiên bản 1/2/3</t>
+  </si>
+  <si>
+    <t>Label contract</t>
+  </si>
+  <si>
+    <t>Headline/Description/Social/Email/CTA dùng đúng label Generator</t>
+  </si>
+  <si>
+    <t>Three versions</t>
+  </si>
+  <si>
+    <t>Đầu ra có đúng 3 phiên bản riêng biệt</t>
+  </si>
+  <si>
+    <t>Unicode</t>
+  </si>
+  <si>
+    <t>Không còn mojibake hay lỗi font trong Excel</t>
+  </si>
+  <si>
+    <t>No CTA marker</t>
+  </si>
+  <si>
+    <t>Không xuất hiện CTA: trong output khi type không phải cta</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -99,14 +143,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,71 +485,81 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{372EFC16-8531-44C4-BFCA-5833655BB3E6}">
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="4" width="14" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="72.77734375" customWidth="1"/>
+    <col min="3" max="3" width="12.77734375" customWidth="1"/>
+    <col min="4" max="4" width="32.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" s="3" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:4" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="4" spans="1:4" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:4" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>7</v>
-      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
     </row>
-    <row r="4" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="6" spans="1:4" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>7</v>
-      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>